<commit_message>
chore(data): daily ingest 2026-05-01
NORMAL/UNKNOWN · GDPNow 3.52 · NY 2.52
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780811B1-8793-4D17-A40A-826966F8EC72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6B6D33-172D-44D9-8377-BAE4A7707DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="1980" windowWidth="21600" windowHeight="11175" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="60">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1598,15 +1598,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="5"/>
+    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1618,7 @@
       <c r="H2" s="29"/>
       <c r="I2" s="29"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
       <c r="D3" s="29"/>
@@ -1628,67 +1628,67 @@
       <c r="H3" s="29"/>
       <c r="I3" s="29"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
+    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1706,14 +1706,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1722,7 +1722,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1731,55 +1731,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1797,13 +1797,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1835,14 +1835,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P184"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P185"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.1796875" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -1851,7 +1851,7 @@
       <c r="G2" s="30"/>
       <c r="H2" s="30"/>
     </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
@@ -1863,16 +1863,16 @@
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="33"/>
     </row>
-    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2520,7 +2520,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2541,7 +2541,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2560,7 +2560,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2579,7 +2579,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2638,7 +2638,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2659,7 +2659,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2680,7 +2680,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2701,7 +2701,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2722,7 +2722,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2743,7 +2743,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2764,7 +2764,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2785,7 +2785,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2806,7 +2806,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2825,7 +2825,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2844,7 +2844,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2863,7 +2863,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2882,7 +2882,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2903,7 +2903,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2945,7 +2945,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2966,7 +2966,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2987,7 +2987,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3008,7 +3008,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3029,7 +3029,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3050,7 +3050,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3071,7 +3071,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3090,7 +3090,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3180,7 +3180,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3557,7 +3557,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3746,7 +3746,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3804,7 +3804,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3881,7 +3881,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3914,7 +3914,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3925,7 +3925,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4027,6 +4027,17 @@
       </c>
       <c r="O184">
         <v>2.81</v>
+      </c>
+    </row>
+    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A185" s="2">
+        <v>46143</v>
+      </c>
+      <c r="N185">
+        <v>2.35</v>
+      </c>
+      <c r="O185">
+        <v>2.52</v>
       </c>
     </row>
   </sheetData>
@@ -4050,18 +4061,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I184"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I185"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -4070,7 +4081,7 @@
       <c r="G2" s="30"/>
       <c r="H2" s="30"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
@@ -4082,16 +4093,16 @@
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="33"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4108,7 +4119,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4119,7 +4130,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4130,7 +4141,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4141,7 +4152,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4152,7 +4163,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4163,7 +4174,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4174,7 +4185,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4185,7 +4196,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4196,7 +4207,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4207,7 +4218,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4218,7 +4229,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4229,7 +4240,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4240,7 +4251,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4254,7 +4265,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4268,7 +4279,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4282,7 +4293,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4296,7 +4307,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4310,7 +4321,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4324,7 +4335,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4338,7 +4349,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4352,7 +4363,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4366,7 +4377,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4380,7 +4391,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4391,7 +4402,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4402,7 +4413,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4413,7 +4424,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4427,7 +4438,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4441,7 +4452,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4455,7 +4466,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4469,7 +4480,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4483,7 +4494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4497,7 +4508,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4511,7 +4522,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4525,7 +4536,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4539,7 +4550,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4553,7 +4564,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4564,7 +4575,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4575,7 +4586,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4586,7 +4597,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4597,7 +4608,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4611,7 +4622,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4625,7 +4636,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4639,7 +4650,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4653,7 +4664,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4667,7 +4678,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4681,7 +4692,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4695,7 +4706,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4709,7 +4720,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4723,7 +4734,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4734,7 +4745,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4745,7 +4756,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4756,7 +4767,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4767,7 +4778,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4781,7 +4792,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4795,7 +4806,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4809,7 +4820,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4823,7 +4834,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4837,7 +4848,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4854,7 +4865,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4871,7 +4882,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4888,7 +4899,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4905,7 +4916,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -4920,7 +4931,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -4935,7 +4946,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -4950,7 +4961,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -4965,7 +4976,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -4982,7 +4993,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -4999,7 +5010,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5013,7 +5024,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5027,7 +5038,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5044,7 +5055,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5061,7 +5072,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5078,7 +5089,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5095,7 +5106,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5112,7 +5123,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5127,7 +5138,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5142,7 +5153,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5157,7 +5168,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5172,7 +5183,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5189,7 +5200,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5206,7 +5217,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5223,7 +5234,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5240,7 +5251,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5257,7 +5268,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5274,7 +5285,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5291,7 +5302,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5308,7 +5319,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5325,7 +5336,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5340,7 +5351,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5355,7 +5366,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5370,7 +5381,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5385,7 +5396,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5402,7 +5413,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5419,7 +5430,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5436,7 +5447,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5450,7 +5461,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5464,7 +5475,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5478,7 +5489,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5492,7 +5503,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5507,7 +5518,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5522,7 +5533,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5537,7 +5548,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5550,7 +5561,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5563,7 +5574,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5576,7 +5587,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5589,7 +5600,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5604,7 +5615,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5619,7 +5630,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5634,7 +5645,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5649,7 +5660,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5663,7 +5674,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5677,7 +5688,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5691,7 +5702,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5705,7 +5716,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5719,7 +5730,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5730,7 +5741,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5741,7 +5752,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5752,7 +5763,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5766,7 +5777,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5780,7 +5791,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5794,7 +5805,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5808,7 +5819,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5822,7 +5833,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5836,7 +5847,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5850,7 +5861,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5864,7 +5875,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5878,7 +5889,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5892,7 +5903,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5903,7 +5914,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5914,7 +5925,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -5925,7 +5936,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -5939,7 +5950,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -5953,7 +5964,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -5967,7 +5978,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -5982,7 +5993,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -5997,7 +6008,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6011,7 +6022,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6026,7 +6037,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6041,7 +6052,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6056,7 +6067,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6071,7 +6082,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6084,7 +6095,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6097,7 +6108,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6110,7 +6121,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6125,7 +6136,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6140,7 +6151,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6155,7 +6166,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6169,7 +6180,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6183,7 +6194,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6197,7 +6208,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6211,7 +6222,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6225,7 +6236,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6239,7 +6250,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6253,7 +6264,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6267,7 +6278,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6281,7 +6292,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6295,7 +6306,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6312,7 +6323,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6326,7 +6337,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6340,7 +6351,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6354,7 +6365,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6368,7 +6379,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6382,7 +6393,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6396,7 +6407,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6410,7 +6421,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6424,7 +6435,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6438,7 +6449,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6452,7 +6463,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6466,7 +6477,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6480,7 +6491,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6491,7 +6502,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6502,7 +6513,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6516,7 +6527,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6530,7 +6541,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6544,7 +6555,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6558,7 +6569,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6572,7 +6583,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6586,7 +6597,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6598,6 +6609,20 @@
       </c>
       <c r="D184">
         <v>2.81</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" s="2">
+        <v>46143</v>
+      </c>
+      <c r="B185" t="s">
+        <v>59</v>
+      </c>
+      <c r="C185">
+        <v>2.35</v>
+      </c>
+      <c r="D185">
+        <v>2.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-05-08
NORMAL/SLOWING · GDPNow 3.75 · NY 2.59
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6B6D33-172D-44D9-8377-BAE4A7707DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E660451-0F5E-4F62-8986-45B48673E5C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="60">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1598,15 +1598,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1618,7 @@
       <c r="H2" s="29"/>
       <c r="I2" s="29"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
       <c r="D3" s="29"/>
@@ -1628,67 +1628,67 @@
       <c r="H3" s="29"/>
       <c r="I3" s="29"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1706,14 +1706,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1722,7 +1722,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1731,55 +1731,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1797,13 +1797,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1835,14 +1835,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P185"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P186"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -1851,7 +1851,7 @@
       <c r="G2" s="30"/>
       <c r="H2" s="30"/>
     </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
@@ -1863,16 +1863,16 @@
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="33"/>
     </row>
-    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2520,7 +2520,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2541,7 +2541,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2560,7 +2560,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2579,7 +2579,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2638,7 +2638,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2659,7 +2659,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2680,7 +2680,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2701,7 +2701,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2722,7 +2722,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2743,7 +2743,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2764,7 +2764,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2785,7 +2785,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2806,7 +2806,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2825,7 +2825,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2844,7 +2844,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2863,7 +2863,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2882,7 +2882,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2903,7 +2903,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2945,7 +2945,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2966,7 +2966,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2987,7 +2987,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3008,7 +3008,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3029,7 +3029,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3050,7 +3050,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3071,7 +3071,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3090,7 +3090,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3180,7 +3180,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3557,7 +3557,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3746,7 +3746,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3804,7 +3804,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3881,7 +3881,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3914,7 +3914,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3925,7 +3925,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4038,6 +4038,14 @@
       </c>
       <c r="O185">
         <v>2.52</v>
+      </c>
+    </row>
+    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A186" s="2">
+        <v>46150</v>
+      </c>
+      <c r="O186">
+        <v>2.59</v>
       </c>
     </row>
   </sheetData>
@@ -4061,18 +4069,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I185"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I186"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -4081,7 +4089,7 @@
       <c r="G2" s="30"/>
       <c r="H2" s="30"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
@@ -4093,16 +4101,16 @@
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="33"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4119,7 +4127,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4130,7 +4138,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4141,7 +4149,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4152,7 +4160,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4163,7 +4171,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4174,7 +4182,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4185,7 +4193,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4196,7 +4204,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4207,7 +4215,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4218,7 +4226,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4229,7 +4237,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4240,7 +4248,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4251,7 +4259,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4265,7 +4273,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4279,7 +4287,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4293,7 +4301,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4307,7 +4315,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4321,7 +4329,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4335,7 +4343,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4349,7 +4357,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4363,7 +4371,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4377,7 +4385,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4391,7 +4399,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4402,7 +4410,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4413,7 +4421,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4424,7 +4432,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4438,7 +4446,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4452,7 +4460,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4466,7 +4474,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4480,7 +4488,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4494,7 +4502,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4508,7 +4516,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4522,7 +4530,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4536,7 +4544,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4550,7 +4558,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4564,7 +4572,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4575,7 +4583,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4586,7 +4594,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4597,7 +4605,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4608,7 +4616,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4622,7 +4630,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4636,7 +4644,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4650,7 +4658,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4664,7 +4672,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4678,7 +4686,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4692,7 +4700,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4706,7 +4714,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4720,7 +4728,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4734,7 +4742,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4745,7 +4753,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4756,7 +4764,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4767,7 +4775,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4778,7 +4786,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4792,7 +4800,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4806,7 +4814,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4820,7 +4828,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4834,7 +4842,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4848,7 +4856,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4865,7 +4873,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4882,7 +4890,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4899,7 +4907,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4916,7 +4924,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -4931,7 +4939,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -4946,7 +4954,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -4961,7 +4969,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -4976,7 +4984,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -4993,7 +5001,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5010,7 +5018,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5024,7 +5032,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5038,7 +5046,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5055,7 +5063,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5072,7 +5080,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5089,7 +5097,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5106,7 +5114,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5123,7 +5131,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5138,7 +5146,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5153,7 +5161,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5168,7 +5176,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5183,7 +5191,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5200,7 +5208,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5217,7 +5225,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5234,7 +5242,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5251,7 +5259,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5268,7 +5276,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5285,7 +5293,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5302,7 +5310,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5319,7 +5327,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5336,7 +5344,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5351,7 +5359,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5366,7 +5374,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5381,7 +5389,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5396,7 +5404,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5413,7 +5421,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5430,7 +5438,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5447,7 +5455,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5461,7 +5469,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5475,7 +5483,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5489,7 +5497,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5503,7 +5511,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5518,7 +5526,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5533,7 +5541,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5548,7 +5556,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5561,7 +5569,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5574,7 +5582,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5587,7 +5595,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5600,7 +5608,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5615,7 +5623,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5630,7 +5638,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5645,7 +5653,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5660,7 +5668,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5674,7 +5682,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5688,7 +5696,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5702,7 +5710,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5716,7 +5724,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5730,7 +5738,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5741,7 +5749,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5752,7 +5760,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5763,7 +5771,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5777,7 +5785,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5791,7 +5799,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5805,7 +5813,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5819,7 +5827,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5833,7 +5841,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5847,7 +5855,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5861,7 +5869,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5875,7 +5883,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5889,7 +5897,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5903,7 +5911,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5914,7 +5922,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5925,7 +5933,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -5936,7 +5944,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -5950,7 +5958,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -5964,7 +5972,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -5978,7 +5986,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -5993,7 +6001,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6008,7 +6016,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6022,7 +6030,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6037,7 +6045,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6052,7 +6060,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6067,7 +6075,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6082,7 +6090,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6095,7 +6103,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6108,7 +6116,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6121,7 +6129,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6136,7 +6144,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6151,7 +6159,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6166,7 +6174,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6180,7 +6188,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6194,7 +6202,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6208,7 +6216,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6222,7 +6230,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6236,7 +6244,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6250,7 +6258,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6264,7 +6272,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6278,7 +6286,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6292,7 +6300,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6306,7 +6314,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6323,7 +6331,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6337,7 +6345,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6351,7 +6359,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6365,7 +6373,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6379,7 +6387,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6393,7 +6401,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6407,7 +6415,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6421,7 +6429,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6435,7 +6443,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6449,7 +6457,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6463,7 +6471,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6477,7 +6485,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6491,7 +6499,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6502,7 +6510,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6513,7 +6521,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6527,7 +6535,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6541,7 +6549,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6555,7 +6563,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6569,7 +6577,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6583,7 +6591,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6597,7 +6605,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6611,7 +6619,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6623,6 +6631,17 @@
       </c>
       <c r="D185">
         <v>2.52</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A186" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B186" t="s">
+        <v>59</v>
+      </c>
+      <c r="D186">
+        <v>2.59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-05-15
NORMAL/SLOWING · GDPNow 3.99 · NY 2.61
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E660451-0F5E-4F62-8986-45B48673E5C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDAF8CC9-7324-4204-8194-BF676CF32C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="4630" yWindow="1300" windowWidth="14380" windowHeight="8170" firstSheet="1" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="60">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1000,9 +1000,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1014,6 +1011,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1607,26 +1607,26 @@
   <sheetData>
     <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
     </row>
     <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
     </row>
     <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
@@ -1835,7 +1835,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P186"/>
+  <dimension ref="A1:P187"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.1796875" customWidth="1"/>
@@ -1843,31 +1843,31 @@
   <sheetData>
     <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:15" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
+      <c r="D4" s="32"/>
     </row>
     <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
@@ -4046,6 +4046,14 @@
       </c>
       <c r="O186">
         <v>2.59</v>
+      </c>
+    </row>
+    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A187" s="2">
+        <v>46157</v>
+      </c>
+      <c r="O187">
+        <v>2.61</v>
       </c>
     </row>
   </sheetData>
@@ -4069,7 +4077,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I187"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.453125" customWidth="1"/>
@@ -4081,31 +4089,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
+      <c r="D4" s="32"/>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
@@ -6642,6 +6650,17 @@
       </c>
       <c r="D186">
         <v>2.59</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A187" s="2">
+        <v>46157</v>
+      </c>
+      <c r="B187" t="s">
+        <v>59</v>
+      </c>
+      <c r="D187">
+        <v>2.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-05-22
NORMAL/SLOWING · GDPNow 4.26 · NY 2.61
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDAF8CC9-7324-4204-8194-BF676CF32C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF61ADD2-1F5D-4AC7-A373-F9745D57362D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4630" yWindow="1300" windowWidth="14380" windowHeight="8170" firstSheet="1" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="60">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1598,15 +1598,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="5"/>
+    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1618,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1628,67 +1628,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
+    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1706,14 +1706,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1722,7 +1722,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1731,55 +1731,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1797,13 +1797,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1835,14 +1835,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P187"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P188"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.1796875" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1851,7 +1851,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1863,16 +1863,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2520,7 +2520,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2541,7 +2541,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2560,7 +2560,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2579,7 +2579,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2638,7 +2638,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2659,7 +2659,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2680,7 +2680,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2701,7 +2701,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2722,7 +2722,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2743,7 +2743,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2764,7 +2764,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2785,7 +2785,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2806,7 +2806,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2825,7 +2825,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2844,7 +2844,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2863,7 +2863,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2882,7 +2882,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2903,7 +2903,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2945,7 +2945,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2966,7 +2966,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2987,7 +2987,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3008,7 +3008,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3029,7 +3029,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3050,7 +3050,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3071,7 +3071,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3090,7 +3090,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3180,7 +3180,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3557,7 +3557,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3746,7 +3746,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3804,7 +3804,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3881,7 +3881,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3914,7 +3914,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3925,7 +3925,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4048,11 +4048,19 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
       <c r="O187">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A188" s="2">
+        <v>46164</v>
+      </c>
+      <c r="O188">
         <v>2.61</v>
       </c>
     </row>
@@ -4077,18 +4085,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I187"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I188"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4097,7 +4105,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4109,16 +4117,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4135,7 +4143,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4146,7 +4154,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4157,7 +4165,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4168,7 +4176,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4179,7 +4187,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4190,7 +4198,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4201,7 +4209,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4212,7 +4220,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4223,7 +4231,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4234,7 +4242,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4245,7 +4253,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4256,7 +4264,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4267,7 +4275,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4281,7 +4289,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4295,7 +4303,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4309,7 +4317,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4323,7 +4331,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4337,7 +4345,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4351,7 +4359,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4365,7 +4373,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4379,7 +4387,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4393,7 +4401,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4407,7 +4415,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4418,7 +4426,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4429,7 +4437,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4440,7 +4448,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4454,7 +4462,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4468,7 +4476,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4482,7 +4490,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4496,7 +4504,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4510,7 +4518,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4524,7 +4532,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4538,7 +4546,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4552,7 +4560,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4566,7 +4574,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4580,7 +4588,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4591,7 +4599,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4602,7 +4610,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4613,7 +4621,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4624,7 +4632,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4638,7 +4646,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4652,7 +4660,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4666,7 +4674,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4680,7 +4688,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4694,7 +4702,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4708,7 +4716,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4722,7 +4730,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4736,7 +4744,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4750,7 +4758,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4761,7 +4769,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4772,7 +4780,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4783,7 +4791,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4794,7 +4802,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4808,7 +4816,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4822,7 +4830,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4836,7 +4844,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4850,7 +4858,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4864,7 +4872,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4881,7 +4889,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4898,7 +4906,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4915,7 +4923,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4932,7 +4940,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -4947,7 +4955,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -4962,7 +4970,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -4977,7 +4985,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -4992,7 +5000,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5009,7 +5017,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5026,7 +5034,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5040,7 +5048,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5054,7 +5062,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5071,7 +5079,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5088,7 +5096,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5105,7 +5113,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5122,7 +5130,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5139,7 +5147,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5154,7 +5162,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5169,7 +5177,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5184,7 +5192,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5199,7 +5207,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5216,7 +5224,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5233,7 +5241,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5250,7 +5258,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5267,7 +5275,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5284,7 +5292,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5301,7 +5309,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5318,7 +5326,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5335,7 +5343,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5352,7 +5360,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5367,7 +5375,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5382,7 +5390,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5397,7 +5405,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5412,7 +5420,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5429,7 +5437,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5446,7 +5454,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5463,7 +5471,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5477,7 +5485,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5491,7 +5499,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5505,7 +5513,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5519,7 +5527,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5534,7 +5542,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5549,7 +5557,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5564,7 +5572,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5577,7 +5585,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5590,7 +5598,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5603,7 +5611,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5616,7 +5624,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5631,7 +5639,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5646,7 +5654,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5661,7 +5669,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5676,7 +5684,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5690,7 +5698,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5704,7 +5712,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5718,7 +5726,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5732,7 +5740,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5746,7 +5754,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5757,7 +5765,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5768,7 +5776,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5779,7 +5787,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5793,7 +5801,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5807,7 +5815,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5821,7 +5829,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5835,7 +5843,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5849,7 +5857,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5863,7 +5871,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5877,7 +5885,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5891,7 +5899,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5905,7 +5913,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5919,7 +5927,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5930,7 +5938,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5941,7 +5949,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -5952,7 +5960,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -5966,7 +5974,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -5980,7 +5988,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -5994,7 +6002,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6009,7 +6017,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6024,7 +6032,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6038,7 +6046,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6053,7 +6061,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6068,7 +6076,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6083,7 +6091,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6098,7 +6106,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6111,7 +6119,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6124,7 +6132,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6137,7 +6145,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6152,7 +6160,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6167,7 +6175,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6182,7 +6190,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6196,7 +6204,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6210,7 +6218,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6224,7 +6232,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6238,7 +6246,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6252,7 +6260,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6266,7 +6274,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6280,7 +6288,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6294,7 +6302,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6308,7 +6316,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6322,7 +6330,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6339,7 +6347,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6353,7 +6361,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6367,7 +6375,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6381,7 +6389,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6395,7 +6403,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6409,7 +6417,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6423,7 +6431,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6437,7 +6445,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6451,7 +6459,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6465,7 +6473,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6479,7 +6487,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6493,7 +6501,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6507,7 +6515,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6518,7 +6526,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6529,7 +6537,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6543,7 +6551,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6557,7 +6565,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6571,7 +6579,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6585,7 +6593,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6599,7 +6607,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6613,7 +6621,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6627,7 +6635,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6641,7 +6649,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6652,7 +6660,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6660,6 +6668,17 @@
         <v>59</v>
       </c>
       <c r="D187">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B188" t="s">
+        <v>59</v>
+      </c>
+      <c r="D188">
         <v>2.61</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-05-30
NORMAL/SLOWING · GDPNow 3.82 · NY 2.5
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF61ADD2-1F5D-4AC7-A373-F9745D57362D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D4D20A-4DAC-40A6-BDC8-FA63D9A303B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="60">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1598,15 +1598,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1618,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1628,67 +1628,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1706,14 +1706,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1722,7 +1722,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1731,55 +1731,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1797,13 +1797,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1835,14 +1835,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P188"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P189"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1851,7 +1851,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1863,16 +1863,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2520,7 +2520,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2541,7 +2541,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2560,7 +2560,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2579,7 +2579,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2638,7 +2638,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2659,7 +2659,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2680,7 +2680,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2701,7 +2701,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2722,7 +2722,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2743,7 +2743,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2764,7 +2764,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2785,7 +2785,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2806,7 +2806,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2825,7 +2825,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2844,7 +2844,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2863,7 +2863,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2882,7 +2882,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2903,7 +2903,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2945,7 +2945,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2966,7 +2966,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2987,7 +2987,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3008,7 +3008,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3029,7 +3029,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3050,7 +3050,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3071,7 +3071,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3090,7 +3090,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3180,7 +3180,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3557,7 +3557,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3746,7 +3746,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3804,7 +3804,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3881,7 +3881,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3914,7 +3914,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3925,7 +3925,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4048,7 +4048,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4056,12 +4056,20 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
       <c r="O188">
         <v>2.61</v>
+      </c>
+    </row>
+    <row r="189" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A189" s="2">
+        <v>46171</v>
+      </c>
+      <c r="O189">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -4085,18 +4093,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I188"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I189"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4105,7 +4113,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4117,16 +4125,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4143,7 +4151,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4154,7 +4162,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4165,7 +4173,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4176,7 +4184,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4187,7 +4195,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4198,7 +4206,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4209,7 +4217,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4220,7 +4228,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4231,7 +4239,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4242,7 +4250,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4253,7 +4261,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4264,7 +4272,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4275,7 +4283,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4289,7 +4297,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4303,7 +4311,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4317,7 +4325,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4331,7 +4339,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4345,7 +4353,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4359,7 +4367,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4373,7 +4381,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4387,7 +4395,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4401,7 +4409,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4415,7 +4423,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4426,7 +4434,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4437,7 +4445,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4448,7 +4456,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4462,7 +4470,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4476,7 +4484,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4490,7 +4498,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4504,7 +4512,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4518,7 +4526,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4532,7 +4540,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4546,7 +4554,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4560,7 +4568,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4574,7 +4582,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4588,7 +4596,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4599,7 +4607,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4610,7 +4618,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4621,7 +4629,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4632,7 +4640,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4646,7 +4654,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4660,7 +4668,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4674,7 +4682,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4688,7 +4696,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4702,7 +4710,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4716,7 +4724,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4730,7 +4738,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4744,7 +4752,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4758,7 +4766,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4769,7 +4777,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4780,7 +4788,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4791,7 +4799,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4802,7 +4810,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4816,7 +4824,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4830,7 +4838,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4844,7 +4852,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4858,7 +4866,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4872,7 +4880,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4889,7 +4897,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4906,7 +4914,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4923,7 +4931,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4940,7 +4948,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -4955,7 +4963,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -4970,7 +4978,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -4985,7 +4993,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5000,7 +5008,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5017,7 +5025,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5034,7 +5042,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5048,7 +5056,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5062,7 +5070,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5079,7 +5087,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5096,7 +5104,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5113,7 +5121,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5130,7 +5138,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5147,7 +5155,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5162,7 +5170,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5177,7 +5185,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5192,7 +5200,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5207,7 +5215,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5224,7 +5232,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5241,7 +5249,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5258,7 +5266,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5275,7 +5283,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5292,7 +5300,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5309,7 +5317,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5326,7 +5334,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5343,7 +5351,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5360,7 +5368,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5375,7 +5383,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5390,7 +5398,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5405,7 +5413,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5420,7 +5428,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5437,7 +5445,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5454,7 +5462,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5471,7 +5479,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5485,7 +5493,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5499,7 +5507,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5513,7 +5521,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5527,7 +5535,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5542,7 +5550,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5557,7 +5565,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5572,7 +5580,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5585,7 +5593,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5598,7 +5606,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5611,7 +5619,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5624,7 +5632,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5639,7 +5647,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5654,7 +5662,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5669,7 +5677,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5684,7 +5692,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5698,7 +5706,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5712,7 +5720,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5726,7 +5734,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5740,7 +5748,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5754,7 +5762,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5765,7 +5773,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5776,7 +5784,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5787,7 +5795,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5801,7 +5809,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5815,7 +5823,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5829,7 +5837,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5843,7 +5851,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5857,7 +5865,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5871,7 +5879,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5885,7 +5893,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5899,7 +5907,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5913,7 +5921,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5927,7 +5935,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5938,7 +5946,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5949,7 +5957,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -5960,7 +5968,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -5974,7 +5982,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -5988,7 +5996,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6002,7 +6010,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6017,7 +6025,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6032,7 +6040,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6046,7 +6054,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6061,7 +6069,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6076,7 +6084,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6091,7 +6099,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6106,7 +6114,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6119,7 +6127,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6132,7 +6140,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6145,7 +6153,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6160,7 +6168,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6175,7 +6183,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6190,7 +6198,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6204,7 +6212,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6218,7 +6226,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6232,7 +6240,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6246,7 +6254,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6260,7 +6268,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6274,7 +6282,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6288,7 +6296,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6302,7 +6310,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6316,7 +6324,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6330,7 +6338,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6347,7 +6355,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6361,7 +6369,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6375,7 +6383,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6389,7 +6397,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6403,7 +6411,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6417,7 +6425,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6431,7 +6439,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6445,7 +6453,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6459,7 +6467,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6473,7 +6481,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6487,7 +6495,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6501,7 +6509,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6515,7 +6523,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6526,7 +6534,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6537,7 +6545,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6551,7 +6559,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6565,7 +6573,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6579,7 +6587,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6593,7 +6601,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6607,7 +6615,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6621,7 +6629,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6635,7 +6643,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6649,7 +6657,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6660,7 +6668,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6671,7 +6679,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6680,6 +6688,17 @@
       </c>
       <c r="D188">
         <v>2.61</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A189" s="2">
+        <v>46171</v>
+      </c>
+      <c r="B189" t="s">
+        <v>59</v>
+      </c>
+      <c r="D189">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-06-05
NORMAL/SLOWING · GDPNow 3.02 · NY 2.67
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D4D20A-4DAC-40A6-BDC8-FA63D9A303B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF75086-4D2C-493F-BEA1-47B69E46B20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>2026:Q2</t>
+  </si>
+  <si>
+    <t>2026Q3</t>
   </si>
 </sst>
 </file>
@@ -1598,15 +1601,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="5"/>
+    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1621,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1628,67 +1631,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
+    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1697,7 +1700,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1706,14 +1709,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1722,7 +1725,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1731,55 +1734,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1788,7 +1791,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1797,13 +1800,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1835,14 +1838,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P189"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P191"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.1796875" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1851,7 +1854,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1863,16 +1866,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1918,8 +1921,11 @@
       <c r="O6" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1927,7 +1933,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1935,7 +1941,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1943,7 +1949,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1951,7 +1957,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1959,7 +1965,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1967,7 +1973,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1975,7 +1981,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1983,7 +1989,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1991,7 +1997,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -1999,7 +2005,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2007,7 +2013,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2015,7 +2021,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2026,7 +2032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2037,7 +2043,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2048,7 +2054,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2059,7 +2065,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2070,7 +2076,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2081,7 +2087,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2092,7 +2098,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2103,7 +2109,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2114,7 +2120,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2125,7 +2131,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2133,7 +2139,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2141,7 +2147,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2149,7 +2155,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2160,7 +2166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2171,7 +2177,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2182,7 +2188,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2193,7 +2199,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2204,7 +2210,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2215,7 +2221,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2226,7 +2232,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2237,7 +2243,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2248,7 +2254,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2259,7 +2265,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2267,7 +2273,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2275,7 +2281,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2283,7 +2289,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2291,7 +2297,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2302,7 +2308,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2313,7 +2319,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2324,7 +2330,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2335,7 +2341,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2346,7 +2352,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2357,7 +2363,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2368,7 +2374,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2379,7 +2385,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2390,7 +2396,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2398,7 +2404,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2406,7 +2412,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2414,7 +2420,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2422,7 +2428,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2433,7 +2439,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2444,7 +2450,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2455,7 +2461,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2466,7 +2472,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2477,7 +2483,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2488,7 +2494,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2499,7 +2505,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2520,7 +2526,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2541,7 +2547,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2560,7 +2566,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2579,7 +2585,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2598,7 +2604,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2617,7 +2623,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2638,7 +2644,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2659,7 +2665,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2680,7 +2686,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2701,7 +2707,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2722,7 +2728,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2743,7 +2749,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2764,7 +2770,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2785,7 +2791,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2806,7 +2812,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2825,7 +2831,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2844,7 +2850,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2863,7 +2869,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2882,7 +2888,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2903,7 +2909,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2924,7 +2930,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2945,7 +2951,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2966,7 +2972,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2987,7 +2993,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3008,7 +3014,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3029,7 +3035,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3050,7 +3056,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3071,7 +3077,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3090,7 +3096,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3098,7 +3104,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3106,7 +3112,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3114,7 +3120,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3125,7 +3131,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3136,7 +3142,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3147,7 +3153,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3158,7 +3164,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3169,7 +3175,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3180,7 +3186,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3191,7 +3197,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3202,7 +3208,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3213,7 +3219,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3224,7 +3230,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3232,7 +3238,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3240,7 +3246,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3248,7 +3254,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3256,7 +3262,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3267,7 +3273,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3278,7 +3284,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3289,7 +3295,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3300,7 +3306,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3311,7 +3317,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3322,7 +3328,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3333,7 +3339,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3344,7 +3350,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3355,7 +3361,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3363,7 +3369,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3371,7 +3377,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3379,7 +3385,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3390,7 +3396,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3401,7 +3407,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3412,7 +3418,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3423,7 +3429,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3434,7 +3440,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3445,7 +3451,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3456,7 +3462,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3467,7 +3473,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3478,7 +3484,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3489,7 +3495,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3497,7 +3503,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3505,7 +3511,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3513,7 +3519,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3524,7 +3530,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3535,7 +3541,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3546,7 +3552,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3557,7 +3563,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3568,7 +3574,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3579,7 +3585,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3590,7 +3596,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3601,7 +3607,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3612,7 +3618,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3623,7 +3629,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3631,7 +3637,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3639,7 +3645,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3647,7 +3653,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3658,7 +3664,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3669,7 +3675,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3680,7 +3686,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3691,7 +3697,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3702,7 +3708,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3713,7 +3719,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3724,7 +3730,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3735,7 +3741,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3746,7 +3752,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3757,7 +3763,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3768,7 +3774,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3779,7 +3785,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3790,7 +3796,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3804,7 +3810,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3815,7 +3821,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3826,7 +3832,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3837,7 +3843,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3848,7 +3854,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3859,7 +3865,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3870,7 +3876,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3881,7 +3887,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3892,7 +3898,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3903,7 +3909,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3914,7 +3920,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3925,7 +3931,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3936,7 +3942,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3944,7 +3950,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3952,7 +3958,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3963,7 +3969,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3974,7 +3980,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3985,7 +3991,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -3996,7 +4002,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4007,7 +4013,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4018,7 +4024,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4029,7 +4035,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4040,7 +4046,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4048,7 +4054,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4056,7 +4062,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4064,13 +4070,30 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
       <c r="O189">
         <v>2.5</v>
       </c>
+      <c r="P189">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A190" s="2">
+        <v>46178</v>
+      </c>
+      <c r="O190">
+        <v>2.67</v>
+      </c>
+      <c r="P190">
+        <v>2.4700000000000002</v>
+      </c>
+    </row>
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A191" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4093,18 +4116,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I189"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I190"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4113,7 +4136,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4125,16 +4148,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4151,7 +4174,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4162,7 +4185,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4173,7 +4196,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4184,7 +4207,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4195,7 +4218,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4206,7 +4229,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4217,7 +4240,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4228,7 +4251,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4239,7 +4262,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4250,7 +4273,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4261,7 +4284,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4272,7 +4295,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4283,7 +4306,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4297,7 +4320,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4311,7 +4334,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4325,7 +4348,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4339,7 +4362,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4353,7 +4376,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4367,7 +4390,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4381,7 +4404,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4395,7 +4418,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4409,7 +4432,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4423,7 +4446,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4434,7 +4457,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4445,7 +4468,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4456,7 +4479,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4470,7 +4493,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4484,7 +4507,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4498,7 +4521,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4512,7 +4535,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4526,7 +4549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4540,7 +4563,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4554,7 +4577,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4568,7 +4591,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4582,7 +4605,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4596,7 +4619,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4607,7 +4630,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4618,7 +4641,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4629,7 +4652,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4640,7 +4663,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4654,7 +4677,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4668,7 +4691,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4682,7 +4705,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4696,7 +4719,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4710,7 +4733,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4724,7 +4747,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4738,7 +4761,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4752,7 +4775,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4766,7 +4789,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4777,7 +4800,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4788,7 +4811,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4799,7 +4822,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4810,7 +4833,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4824,7 +4847,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4838,7 +4861,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4852,7 +4875,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4866,7 +4889,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4880,7 +4903,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4897,7 +4920,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4914,7 +4937,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4931,7 +4954,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4948,7 +4971,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -4963,7 +4986,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -4978,7 +5001,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -4993,7 +5016,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5008,7 +5031,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5025,7 +5048,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5042,7 +5065,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5056,7 +5079,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5070,7 +5093,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5087,7 +5110,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5104,7 +5127,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5121,7 +5144,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5138,7 +5161,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5155,7 +5178,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5170,7 +5193,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5185,7 +5208,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5200,7 +5223,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5215,7 +5238,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5232,7 +5255,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5249,7 +5272,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5266,7 +5289,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5283,7 +5306,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5300,7 +5323,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5317,7 +5340,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5334,7 +5357,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5351,7 +5374,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5368,7 +5391,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5383,7 +5406,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5398,7 +5421,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5413,7 +5436,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5428,7 +5451,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5445,7 +5468,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5462,7 +5485,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5479,7 +5502,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5493,7 +5516,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5507,7 +5530,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5521,7 +5544,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5535,7 +5558,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5550,7 +5573,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5565,7 +5588,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5580,7 +5603,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5593,7 +5616,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5606,7 +5629,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5619,7 +5642,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5632,7 +5655,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5647,7 +5670,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5662,7 +5685,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5677,7 +5700,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5692,7 +5715,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5706,7 +5729,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5720,7 +5743,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5734,7 +5757,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5748,7 +5771,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5762,7 +5785,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5773,7 +5796,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5784,7 +5807,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5795,7 +5818,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5809,7 +5832,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5823,7 +5846,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5837,7 +5860,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5851,7 +5874,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5865,7 +5888,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5879,7 +5902,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5893,7 +5916,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5907,7 +5930,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5921,7 +5944,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5935,7 +5958,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5946,7 +5969,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5957,7 +5980,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -5968,7 +5991,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -5982,7 +6005,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -5996,7 +6019,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6010,7 +6033,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6025,7 +6048,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6040,7 +6063,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6054,7 +6077,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6069,7 +6092,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6084,7 +6107,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6099,7 +6122,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6114,7 +6137,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6127,7 +6150,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6140,7 +6163,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6153,7 +6176,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6168,7 +6191,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6183,7 +6206,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6198,7 +6221,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6212,7 +6235,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6226,7 +6249,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6240,7 +6263,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6254,7 +6277,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6268,7 +6291,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6282,7 +6305,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6296,7 +6319,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6310,7 +6333,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6324,7 +6347,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6338,7 +6361,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6355,7 +6378,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6369,7 +6392,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6383,7 +6406,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6397,7 +6420,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6411,7 +6434,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6425,7 +6448,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6439,7 +6462,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6453,7 +6476,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6467,7 +6490,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6481,7 +6504,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6495,7 +6518,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6509,7 +6532,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6523,7 +6546,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6534,7 +6557,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6545,7 +6568,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6559,7 +6582,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6573,7 +6596,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6587,7 +6610,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6601,7 +6624,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6615,7 +6638,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6629,7 +6652,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6643,7 +6666,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6657,7 +6680,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6668,7 +6691,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6679,7 +6702,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6690,7 +6713,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6699,6 +6722,23 @@
       </c>
       <c r="D189">
         <v>2.5</v>
+      </c>
+      <c r="E189">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" s="2">
+        <v>46178</v>
+      </c>
+      <c r="B190" t="s">
+        <v>59</v>
+      </c>
+      <c r="D190">
+        <v>2.67</v>
+      </c>
+      <c r="E190">
+        <v>2.4700000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-06-13
NORMAL/SLOWING · GDPNow 3.29 · NY 2.7
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF75086-4D2C-493F-BEA1-47B69E46B20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E9A7E5-00CC-420A-AC2E-41EE41AB8498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="57480" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1601,15 +1601,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1621,7 +1621,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1631,67 +1631,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1700,7 +1700,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1709,14 +1709,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1725,7 +1725,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1734,55 +1734,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1791,7 +1791,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1800,13 +1800,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1839,13 +1839,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
   <dimension ref="A1:P191"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1854,7 +1854,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1866,16 +1866,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2363,7 +2363,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2526,7 +2526,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2547,7 +2547,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2566,7 +2566,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2585,7 +2585,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2604,7 +2604,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2623,7 +2623,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2644,7 +2644,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2665,7 +2665,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2686,7 +2686,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2707,7 +2707,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2728,7 +2728,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2749,7 +2749,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2770,7 +2770,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2791,7 +2791,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2812,7 +2812,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2831,7 +2831,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2850,7 +2850,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2869,7 +2869,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2888,7 +2888,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2909,7 +2909,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2930,7 +2930,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2951,7 +2951,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2972,7 +2972,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2993,7 +2993,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3014,7 +3014,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3035,7 +3035,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3056,7 +3056,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3077,7 +3077,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3096,7 +3096,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3131,7 +3131,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3262,7 +3262,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3306,7 +3306,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3396,7 +3396,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3440,7 +3440,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3495,7 +3495,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3511,7 +3511,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3596,7 +3596,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3719,7 +3719,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3785,7 +3785,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3796,7 +3796,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3810,7 +3810,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3821,7 +3821,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3843,7 +3843,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3887,7 +3887,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3898,7 +3898,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3909,7 +3909,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3920,7 +3920,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3931,7 +3931,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3942,7 +3942,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4002,7 +4002,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4046,7 +4046,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4062,7 +4062,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4070,7 +4070,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4092,8 +4092,16 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A191" s="2"/>
+    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A191" s="2">
+        <v>46185</v>
+      </c>
+      <c r="O191">
+        <v>2.7</v>
+      </c>
+      <c r="P191">
+        <v>2.46</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4116,18 +4124,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I190"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I191"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4136,7 +4144,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4148,16 +4156,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4174,7 +4182,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4185,7 +4193,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4196,7 +4204,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4207,7 +4215,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4218,7 +4226,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4229,7 +4237,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4240,7 +4248,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4251,7 +4259,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4262,7 +4270,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4273,7 +4281,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4284,7 +4292,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4295,7 +4303,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4306,7 +4314,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4320,7 +4328,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4334,7 +4342,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4348,7 +4356,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4362,7 +4370,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4376,7 +4384,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4390,7 +4398,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4404,7 +4412,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4418,7 +4426,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4432,7 +4440,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4446,7 +4454,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4457,7 +4465,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4468,7 +4476,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4479,7 +4487,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4493,7 +4501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4507,7 +4515,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4521,7 +4529,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4535,7 +4543,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4549,7 +4557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4563,7 +4571,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4577,7 +4585,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4591,7 +4599,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4605,7 +4613,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4619,7 +4627,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4630,7 +4638,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4641,7 +4649,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4652,7 +4660,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4663,7 +4671,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4677,7 +4685,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4691,7 +4699,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4705,7 +4713,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4719,7 +4727,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4733,7 +4741,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4747,7 +4755,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4761,7 +4769,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4775,7 +4783,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4789,7 +4797,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4800,7 +4808,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4811,7 +4819,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4822,7 +4830,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4833,7 +4841,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4847,7 +4855,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4861,7 +4869,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4875,7 +4883,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4889,7 +4897,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4903,7 +4911,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4920,7 +4928,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4937,7 +4945,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4954,7 +4962,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4971,7 +4979,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -4986,7 +4994,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5001,7 +5009,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5016,7 +5024,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5031,7 +5039,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5048,7 +5056,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5065,7 +5073,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5079,7 +5087,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5093,7 +5101,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5110,7 +5118,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5127,7 +5135,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5144,7 +5152,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5161,7 +5169,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5178,7 +5186,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5193,7 +5201,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5208,7 +5216,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5223,7 +5231,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5238,7 +5246,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5255,7 +5263,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5272,7 +5280,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5289,7 +5297,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5306,7 +5314,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5323,7 +5331,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5340,7 +5348,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5357,7 +5365,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5374,7 +5382,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5391,7 +5399,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5406,7 +5414,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5421,7 +5429,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5436,7 +5444,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5451,7 +5459,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5468,7 +5476,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5485,7 +5493,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5502,7 +5510,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5516,7 +5524,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5530,7 +5538,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5544,7 +5552,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5558,7 +5566,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5573,7 +5581,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5588,7 +5596,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5603,7 +5611,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5616,7 +5624,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5629,7 +5637,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5642,7 +5650,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5655,7 +5663,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5670,7 +5678,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5685,7 +5693,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5700,7 +5708,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5715,7 +5723,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5729,7 +5737,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5743,7 +5751,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5757,7 +5765,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5771,7 +5779,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5785,7 +5793,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5796,7 +5804,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5807,7 +5815,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5818,7 +5826,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5832,7 +5840,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5846,7 +5854,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5860,7 +5868,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5874,7 +5882,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5888,7 +5896,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5902,7 +5910,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5916,7 +5924,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5930,7 +5938,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5944,7 +5952,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5958,7 +5966,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5969,7 +5977,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5980,7 +5988,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -5991,7 +5999,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6005,7 +6013,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6019,7 +6027,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6033,7 +6041,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6048,7 +6056,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6063,7 +6071,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6077,7 +6085,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6092,7 +6100,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6107,7 +6115,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6122,7 +6130,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6137,7 +6145,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6150,7 +6158,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6163,7 +6171,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6176,7 +6184,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6191,7 +6199,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6206,7 +6214,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6221,7 +6229,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6235,7 +6243,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6249,7 +6257,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6263,7 +6271,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6277,7 +6285,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6291,7 +6299,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6305,7 +6313,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6319,7 +6327,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6333,7 +6341,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6347,7 +6355,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6361,7 +6369,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6378,7 +6386,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6392,7 +6400,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6406,7 +6414,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6420,7 +6428,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6434,7 +6442,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6448,7 +6456,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6462,7 +6470,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6476,7 +6484,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6490,7 +6498,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6504,7 +6512,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6518,7 +6526,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6532,7 +6540,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6546,7 +6554,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6557,7 +6565,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6568,7 +6576,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6582,7 +6590,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6596,7 +6604,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6610,7 +6618,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6624,7 +6632,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6638,7 +6646,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6652,7 +6660,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6666,7 +6674,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6680,7 +6688,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6691,7 +6699,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6702,7 +6710,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6713,7 +6721,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6727,7 +6735,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6739,6 +6747,20 @@
       </c>
       <c r="E190">
         <v>2.4700000000000002</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A191" s="2">
+        <v>46185</v>
+      </c>
+      <c r="B191" t="s">
+        <v>59</v>
+      </c>
+      <c r="D191">
+        <v>2.7</v>
+      </c>
+      <c r="E191">
+        <v>2.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-06-19
NORMAL/SLOWING · GDPNow 3.04 · NY 2.68
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E9A7E5-00CC-420A-AC2E-41EE41AB8498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23DAA14-D95F-4A8D-8458-4DA42E7F5F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1003,6 +1003,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1014,9 +1017,6 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1610,26 +1610,26 @@
   <sheetData>
     <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
     </row>
     <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
@@ -1838,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P191"/>
+  <dimension ref="A1:P192"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.1796875" customWidth="1"/>
@@ -1846,31 +1846,31 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
+      <c r="D4" s="33"/>
     </row>
     <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
@@ -4101,6 +4101,17 @@
       </c>
       <c r="P191">
         <v>2.46</v>
+      </c>
+    </row>
+    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A192" s="2">
+        <v>46192</v>
+      </c>
+      <c r="O192">
+        <v>2.68</v>
+      </c>
+      <c r="P192">
+        <v>2.4500000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -4124,7 +4135,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I191"/>
+  <dimension ref="A1:I192"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.453125" customWidth="1"/>
@@ -4136,31 +4147,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
+      <c r="D4" s="33"/>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
@@ -6761,6 +6772,20 @@
       </c>
       <c r="E191">
         <v>2.46</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A192" s="2">
+        <v>46192</v>
+      </c>
+      <c r="B192" t="s">
+        <v>59</v>
+      </c>
+      <c r="D192">
+        <v>2.68</v>
+      </c>
+      <c r="E192">
+        <v>2.4500000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-06-26
NORMAL/SLOWING · GDPNow 2.54 · NY 2.7
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23DAA14-D95F-4A8D-8458-4DA42E7F5F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46DCEFC5-D0FC-4E1F-B30A-D911F90C7CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1003,9 +1003,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1017,6 +1014,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1601,97 +1601,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="5"/>
+    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="29" t="s">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-    </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-    </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+    </row>
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+    </row>
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
+    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1700,7 +1700,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1709,14 +1709,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1725,7 +1725,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1734,55 +1734,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1791,7 +1791,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1800,13 +1800,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1838,44 +1838,44 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P192"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P193"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.1796875" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-    </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="31" t="s">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+    </row>
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-    </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="33" t="s">
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+    </row>
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
-    </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="32"/>
+    </row>
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2363,7 +2363,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2526,7 +2526,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2547,7 +2547,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2566,7 +2566,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2585,7 +2585,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2604,7 +2604,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2623,7 +2623,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2644,7 +2644,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2665,7 +2665,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2686,7 +2686,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2707,7 +2707,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2728,7 +2728,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2749,7 +2749,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2770,7 +2770,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2791,7 +2791,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2812,7 +2812,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2831,7 +2831,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2850,7 +2850,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2869,7 +2869,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2888,7 +2888,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2909,7 +2909,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2930,7 +2930,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2951,7 +2951,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2972,7 +2972,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2993,7 +2993,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3014,7 +3014,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3035,7 +3035,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3056,7 +3056,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3077,7 +3077,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3096,7 +3096,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3131,7 +3131,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3262,7 +3262,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3306,7 +3306,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3396,7 +3396,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3440,7 +3440,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3495,7 +3495,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3511,7 +3511,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3596,7 +3596,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3719,7 +3719,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3785,7 +3785,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3796,7 +3796,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3810,7 +3810,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3821,7 +3821,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3843,7 +3843,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3887,7 +3887,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3898,7 +3898,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3909,7 +3909,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3920,7 +3920,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3931,7 +3931,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3942,7 +3942,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4002,7 +4002,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4046,7 +4046,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4062,7 +4062,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4070,7 +4070,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -4112,6 +4112,17 @@
       </c>
       <c r="P192">
         <v>2.4500000000000002</v>
+      </c>
+    </row>
+    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A193" s="2">
+        <v>46199</v>
+      </c>
+      <c r="O193">
+        <v>2.7</v>
+      </c>
+      <c r="P193">
+        <v>2.42</v>
       </c>
     </row>
   </sheetData>
@@ -4135,48 +4146,48 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I192"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I193"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-    </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="31" t="s">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+    </row>
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-    </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="33" t="s">
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+    </row>
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
-    </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="32"/>
+    </row>
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4193,7 +4204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4204,7 +4215,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4215,7 +4226,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4226,7 +4237,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4237,7 +4248,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4248,7 +4259,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4259,7 +4270,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4270,7 +4281,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4281,7 +4292,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4292,7 +4303,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4303,7 +4314,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4314,7 +4325,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4325,7 +4336,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4339,7 +4350,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4353,7 +4364,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4367,7 +4378,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4381,7 +4392,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4395,7 +4406,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4409,7 +4420,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4423,7 +4434,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4437,7 +4448,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4451,7 +4462,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4465,7 +4476,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4476,7 +4487,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4487,7 +4498,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4498,7 +4509,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4512,7 +4523,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4526,7 +4537,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4540,7 +4551,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4554,7 +4565,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4568,7 +4579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4582,7 +4593,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4596,7 +4607,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4610,7 +4621,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4624,7 +4635,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4638,7 +4649,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4649,7 +4660,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4660,7 +4671,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4671,7 +4682,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4682,7 +4693,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4696,7 +4707,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4710,7 +4721,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4724,7 +4735,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4738,7 +4749,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4752,7 +4763,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4766,7 +4777,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4780,7 +4791,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4794,7 +4805,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4808,7 +4819,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4819,7 +4830,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4830,7 +4841,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4841,7 +4852,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4852,7 +4863,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4866,7 +4877,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4880,7 +4891,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4894,7 +4905,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4908,7 +4919,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4922,7 +4933,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4939,7 +4950,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -4956,7 +4967,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -4973,7 +4984,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -4990,7 +5001,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -5005,7 +5016,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5020,7 +5031,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5035,7 +5046,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5050,7 +5061,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5067,7 +5078,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5084,7 +5095,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5098,7 +5109,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5112,7 +5123,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5129,7 +5140,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5146,7 +5157,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5163,7 +5174,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5180,7 +5191,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5197,7 +5208,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5212,7 +5223,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5227,7 +5238,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5242,7 +5253,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5257,7 +5268,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5274,7 +5285,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5291,7 +5302,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5308,7 +5319,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5325,7 +5336,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5342,7 +5353,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5359,7 +5370,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5376,7 +5387,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5393,7 +5404,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5410,7 +5421,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5425,7 +5436,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5440,7 +5451,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5455,7 +5466,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5470,7 +5481,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5487,7 +5498,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5504,7 +5515,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5521,7 +5532,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5535,7 +5546,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5549,7 +5560,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5563,7 +5574,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5577,7 +5588,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5592,7 +5603,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5607,7 +5618,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5622,7 +5633,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5635,7 +5646,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5648,7 +5659,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5661,7 +5672,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5674,7 +5685,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5689,7 +5700,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5704,7 +5715,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5719,7 +5730,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5734,7 +5745,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5748,7 +5759,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5762,7 +5773,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5776,7 +5787,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5790,7 +5801,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5804,7 +5815,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5815,7 +5826,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5826,7 +5837,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5837,7 +5848,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5851,7 +5862,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5865,7 +5876,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5879,7 +5890,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5893,7 +5904,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5907,7 +5918,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5921,7 +5932,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5935,7 +5946,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -5949,7 +5960,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -5963,7 +5974,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -5977,7 +5988,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -5988,7 +5999,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -5999,7 +6010,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -6010,7 +6021,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6024,7 +6035,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6038,7 +6049,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6052,7 +6063,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6067,7 +6078,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6082,7 +6093,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6096,7 +6107,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6111,7 +6122,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6126,7 +6137,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6141,7 +6152,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6156,7 +6167,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6169,7 +6180,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6182,7 +6193,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6195,7 +6206,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6210,7 +6221,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6225,7 +6236,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6240,7 +6251,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6254,7 +6265,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6268,7 +6279,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6282,7 +6293,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6296,7 +6307,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6310,7 +6321,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6324,7 +6335,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6338,7 +6349,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6352,7 +6363,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6366,7 +6377,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6380,7 +6391,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6397,7 +6408,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6411,7 +6422,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6425,7 +6436,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6439,7 +6450,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6453,7 +6464,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6467,7 +6478,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6481,7 +6492,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6495,7 +6506,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6509,7 +6520,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6523,7 +6534,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6537,7 +6548,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6551,7 +6562,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6565,7 +6576,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6576,7 +6587,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6587,7 +6598,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6601,7 +6612,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6615,7 +6626,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6629,7 +6640,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6643,7 +6654,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6657,7 +6668,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6671,7 +6682,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6685,7 +6696,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6699,7 +6710,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6710,7 +6721,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6721,7 +6732,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6732,7 +6743,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6746,7 +6757,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6760,7 +6771,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -6774,7 +6785,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -6786,6 +6797,20 @@
       </c>
       <c r="E192">
         <v>2.4500000000000002</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" s="2">
+        <v>46199</v>
+      </c>
+      <c r="B193" t="s">
+        <v>59</v>
+      </c>
+      <c r="D193">
+        <v>2.7</v>
+      </c>
+      <c r="E193">
+        <v>2.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-07-03
NORMAL/SLOWING · GDPNow 1.19 · NY 2.74
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46DCEFC5-D0FC-4E1F-B30A-D911F90C7CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B396E225-D560-4469-9CED-A2BB974DB2AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1838,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P193"/>
+  <dimension ref="A1:P194"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -4123,6 +4123,17 @@
       </c>
       <c r="P193">
         <v>2.42</v>
+      </c>
+    </row>
+    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A194" s="2">
+        <v>46206</v>
+      </c>
+      <c r="O194">
+        <v>2.74</v>
+      </c>
+      <c r="P194">
+        <v>2.37</v>
       </c>
     </row>
   </sheetData>
@@ -4146,7 +4157,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I193"/>
+  <dimension ref="A1:I194"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -6811,6 +6822,20 @@
       </c>
       <c r="E193">
         <v>2.42</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" s="2">
+        <v>46206</v>
+      </c>
+      <c r="B194" t="s">
+        <v>59</v>
+      </c>
+      <c r="D194">
+        <v>2.74</v>
+      </c>
+      <c r="E194">
+        <v>2.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-07-10
NORMAL/SLOWING · GDPNow 1.26 · NY 2.73
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B396E225-D560-4469-9CED-A2BB974DB2AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BE0C48-C84F-4D99-BE8C-F3A29CA83188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1838,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P194"/>
+  <dimension ref="A1:P195"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -4134,6 +4134,17 @@
       </c>
       <c r="P194">
         <v>2.37</v>
+      </c>
+    </row>
+    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A195" s="2">
+        <v>46213</v>
+      </c>
+      <c r="O195">
+        <v>2.73</v>
+      </c>
+      <c r="P195">
+        <v>2.36</v>
       </c>
     </row>
   </sheetData>
@@ -4157,7 +4168,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I194"/>
+  <dimension ref="A1:I195"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -6836,6 +6847,20 @@
       </c>
       <c r="E194">
         <v>2.37</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" s="2">
+        <v>46213</v>
+      </c>
+      <c r="B195" t="s">
+        <v>59</v>
+      </c>
+      <c r="D195">
+        <v>2.73</v>
+      </c>
+      <c r="E195">
+        <v>2.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-07-17
NORMAL/SLOWING · GDPNow 1.68 · NY 2.8
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BE0C48-C84F-4D99-BE8C-F3A29CA83188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB486EE0-7B03-4803-9A41-697334EB6450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1003,6 +1003,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1014,9 +1017,6 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1610,26 +1610,26 @@
   <sheetData>
     <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
     </row>
     <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
@@ -1838,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P195"/>
+  <dimension ref="A1:P196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -1846,31 +1846,31 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
+      <c r="D4" s="33"/>
     </row>
     <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -4145,6 +4145,17 @@
       </c>
       <c r="P195">
         <v>2.36</v>
+      </c>
+    </row>
+    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A196" s="2">
+        <v>46220</v>
+      </c>
+      <c r="O196">
+        <v>2.8</v>
+      </c>
+      <c r="P196">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -4168,7 +4179,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I195"/>
+  <dimension ref="A1:I196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -4180,31 +4191,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
+      <c r="D4" s="33"/>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -6861,6 +6872,20 @@
       </c>
       <c r="E195">
         <v>2.36</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" s="2">
+        <v>46220</v>
+      </c>
+      <c r="B196" t="s">
+        <v>59</v>
+      </c>
+      <c r="D196">
+        <v>2.8</v>
+      </c>
+      <c r="E196">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-07-24
NORMAL/SLOWING · GDPNow 1.68 · NY 2.8
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB486EE0-7B03-4803-9A41-697334EB6450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB27510E-86A3-4CCB-B61B-2EAD9DCBB89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="61">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1003,9 +1003,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1017,6 +1014,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1610,26 +1610,26 @@
   <sheetData>
     <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
     </row>
     <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
     </row>
     <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
@@ -1838,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P196"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -1846,31 +1846,31 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
+      <c r="D4" s="32"/>
     </row>
     <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -4155,6 +4155,17 @@
         <v>2.8</v>
       </c>
       <c r="P196">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A197" s="2">
+        <v>46227</v>
+      </c>
+      <c r="O197">
+        <v>2.8</v>
+      </c>
+      <c r="P197">
         <v>2.6</v>
       </c>
     </row>
@@ -4179,7 +4190,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I196"/>
+  <dimension ref="A1:I197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -4191,31 +4202,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
+      <c r="D4" s="32"/>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -6885,6 +6896,20 @@
         <v>2.8</v>
       </c>
       <c r="E196">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" s="2">
+        <v>46227</v>
+      </c>
+      <c r="B197" t="s">
+        <v>59</v>
+      </c>
+      <c r="D197">
+        <v>2.8</v>
+      </c>
+      <c r="E197">
         <v>2.6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-07-31
NORMAL/SLOWING · GDPNow 4.95 · NY 2.52
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB27510E-86A3-4CCB-B61B-2EAD9DCBB89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0174EF66-3B42-4D05-85A8-2C037002A395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>2026Q3</t>
+  </si>
+  <si>
+    <t>2026:Q3</t>
   </si>
 </sst>
 </file>
@@ -1601,15 +1604,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1621,7 +1624,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1631,67 +1634,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1700,7 +1703,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1709,14 +1712,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1725,7 +1728,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1734,55 +1737,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1791,7 +1794,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1800,13 +1803,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1838,14 +1841,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P197"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P198"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1854,7 +1857,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1866,16 +1869,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1925,7 +1928,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1933,7 +1936,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1941,7 +1944,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1949,7 +1952,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1957,7 +1960,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1965,7 +1968,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1973,7 +1976,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1981,7 +1984,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1989,7 +1992,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -1997,7 +2000,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2005,7 +2008,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2013,7 +2016,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2021,7 +2024,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2032,7 +2035,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2043,7 +2046,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2054,7 +2057,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2065,7 +2068,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2087,7 +2090,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2098,7 +2101,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2109,7 +2112,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2120,7 +2123,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2131,7 +2134,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2139,7 +2142,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2147,7 +2150,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2155,7 +2158,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2166,7 +2169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2177,7 +2180,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2188,7 +2191,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2199,7 +2202,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2210,7 +2213,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2221,7 +2224,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2232,7 +2235,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2243,7 +2246,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2265,7 +2268,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2273,7 +2276,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2281,7 +2284,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2289,7 +2292,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2297,7 +2300,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2308,7 +2311,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2319,7 +2322,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2330,7 +2333,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2341,7 +2344,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2352,7 +2355,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2363,7 +2366,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2374,7 +2377,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2385,7 +2388,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2396,7 +2399,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2404,7 +2407,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2412,7 +2415,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2420,7 +2423,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2428,7 +2431,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2439,7 +2442,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2450,7 +2453,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2461,7 +2464,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2472,7 +2475,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2483,7 +2486,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2494,7 +2497,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2505,7 +2508,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2526,7 +2529,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2547,7 +2550,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2566,7 +2569,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2585,7 +2588,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2604,7 +2607,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2623,7 +2626,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2644,7 +2647,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2665,7 +2668,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2686,7 +2689,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2707,7 +2710,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2728,7 +2731,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2749,7 +2752,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2770,7 +2773,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2791,7 +2794,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2812,7 +2815,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2831,7 +2834,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2850,7 +2853,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2869,7 +2872,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2888,7 +2891,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2909,7 +2912,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2930,7 +2933,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2951,7 +2954,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2972,7 +2975,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2993,7 +2996,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3014,7 +3017,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3035,7 +3038,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3056,7 +3059,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3077,7 +3080,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3096,7 +3099,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3104,7 +3107,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3112,7 +3115,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3120,7 +3123,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3142,7 +3145,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3153,7 +3156,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3164,7 +3167,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3175,7 +3178,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3186,7 +3189,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3197,7 +3200,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3208,7 +3211,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3219,7 +3222,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3230,7 +3233,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3238,7 +3241,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3246,7 +3249,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3254,7 +3257,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3262,7 +3265,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3273,7 +3276,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3284,7 +3287,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3295,7 +3298,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3306,7 +3309,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3317,7 +3320,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3328,7 +3331,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3339,7 +3342,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3350,7 +3353,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3361,7 +3364,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3369,7 +3372,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3377,7 +3380,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3385,7 +3388,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3396,7 +3399,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3407,7 +3410,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3418,7 +3421,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3429,7 +3432,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3440,7 +3443,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3451,7 +3454,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3462,7 +3465,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3473,7 +3476,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3484,7 +3487,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3495,7 +3498,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3503,7 +3506,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3511,7 +3514,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3519,7 +3522,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3530,7 +3533,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3541,7 +3544,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3552,7 +3555,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3563,7 +3566,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3574,7 +3577,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3585,7 +3588,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3596,7 +3599,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3607,7 +3610,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3618,7 +3621,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3629,7 +3632,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3637,7 +3640,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3645,7 +3648,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3653,7 +3656,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3664,7 +3667,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3675,7 +3678,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3686,7 +3689,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3697,7 +3700,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3708,7 +3711,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3719,7 +3722,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3730,7 +3733,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3741,7 +3744,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3752,7 +3755,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3763,7 +3766,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3774,7 +3777,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3785,7 +3788,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3796,7 +3799,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3810,7 +3813,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3821,7 +3824,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3832,7 +3835,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3843,7 +3846,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3854,7 +3857,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3865,7 +3868,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3876,7 +3879,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3887,7 +3890,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3898,7 +3901,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3909,7 +3912,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3920,7 +3923,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3931,7 +3934,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3942,7 +3945,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3950,7 +3953,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3958,7 +3961,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3969,7 +3972,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3980,7 +3983,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3991,7 +3994,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4002,7 +4005,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4013,7 +4016,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4024,7 +4027,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4035,7 +4038,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4046,7 +4049,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4054,7 +4057,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4062,7 +4065,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4070,7 +4073,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4081,7 +4084,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4092,7 +4095,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -4103,7 +4106,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -4114,7 +4117,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -4125,7 +4128,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -4136,7 +4139,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -4147,7 +4150,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -4158,15 +4161,26 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
       <c r="O197">
-        <v>2.8</v>
+        <v>2.82</v>
       </c>
       <c r="P197">
-        <v>2.6</v>
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A198" s="2">
+        <v>46234</v>
+      </c>
+      <c r="O198">
+        <v>2.85</v>
+      </c>
+      <c r="P198">
+        <v>2.52</v>
       </c>
     </row>
   </sheetData>
@@ -4190,18 +4204,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I197"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I198"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4210,7 +4224,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4222,16 +4236,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4248,7 +4262,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4259,7 +4273,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4270,7 +4284,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4281,7 +4295,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4292,7 +4306,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4303,7 +4317,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4314,7 +4328,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4325,7 +4339,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4336,7 +4350,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4347,7 +4361,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4358,7 +4372,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4369,7 +4383,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4380,7 +4394,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4394,7 +4408,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4408,7 +4422,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4422,7 +4436,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4436,7 +4450,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4450,7 +4464,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4464,7 +4478,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4478,7 +4492,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4492,7 +4506,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4506,7 +4520,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4520,7 +4534,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4531,7 +4545,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4542,7 +4556,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4553,7 +4567,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4567,7 +4581,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4581,7 +4595,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4595,7 +4609,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4609,7 +4623,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4623,7 +4637,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4637,7 +4651,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4651,7 +4665,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4665,7 +4679,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4679,7 +4693,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4693,7 +4707,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4704,7 +4718,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4715,7 +4729,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4726,7 +4740,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4737,7 +4751,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4751,7 +4765,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4765,7 +4779,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4779,7 +4793,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4793,7 +4807,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4807,7 +4821,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4821,7 +4835,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4835,7 +4849,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4849,7 +4863,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4863,7 +4877,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4874,7 +4888,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4885,7 +4899,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4896,7 +4910,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4907,7 +4921,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4921,7 +4935,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4935,7 +4949,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4949,7 +4963,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4963,7 +4977,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4977,7 +4991,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -4994,7 +5008,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -5011,7 +5025,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -5028,7 +5042,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -5045,7 +5059,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -5060,7 +5074,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5075,7 +5089,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5090,7 +5104,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5105,7 +5119,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5122,7 +5136,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5139,7 +5153,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5153,7 +5167,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5167,7 +5181,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5184,7 +5198,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5201,7 +5215,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5218,7 +5232,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5235,7 +5249,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5252,7 +5266,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5267,7 +5281,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5282,7 +5296,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5297,7 +5311,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5312,7 +5326,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5329,7 +5343,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5346,7 +5360,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5363,7 +5377,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5380,7 +5394,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5397,7 +5411,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5414,7 +5428,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5431,7 +5445,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5448,7 +5462,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5465,7 +5479,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5480,7 +5494,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5495,7 +5509,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5510,7 +5524,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5525,7 +5539,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5542,7 +5556,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5559,7 +5573,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5576,7 +5590,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5590,7 +5604,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5604,7 +5618,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5618,7 +5632,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5632,7 +5646,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5647,7 +5661,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5662,7 +5676,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5677,7 +5691,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5690,7 +5704,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5703,7 +5717,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5716,7 +5730,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5729,7 +5743,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5744,7 +5758,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5759,7 +5773,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5774,7 +5788,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5789,7 +5803,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5803,7 +5817,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5817,7 +5831,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5831,7 +5845,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5845,7 +5859,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5859,7 +5873,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5870,7 +5884,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5881,7 +5895,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5892,7 +5906,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5906,7 +5920,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5920,7 +5934,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5934,7 +5948,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5948,7 +5962,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5962,7 +5976,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5976,7 +5990,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -5990,7 +6004,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -6004,7 +6018,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -6018,7 +6032,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -6032,7 +6046,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -6043,7 +6057,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -6054,7 +6068,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -6065,7 +6079,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6079,7 +6093,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6093,7 +6107,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6107,7 +6121,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6122,7 +6136,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6137,7 +6151,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6151,7 +6165,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6166,7 +6180,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6181,7 +6195,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6196,7 +6210,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6211,7 +6225,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6224,7 +6238,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6237,7 +6251,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6250,7 +6264,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6265,7 +6279,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6280,7 +6294,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6295,7 +6309,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6309,7 +6323,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6323,7 +6337,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6337,7 +6351,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6351,7 +6365,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6365,7 +6379,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6379,7 +6393,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6393,7 +6407,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6407,7 +6421,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6421,7 +6435,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6435,7 +6449,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6452,7 +6466,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6466,7 +6480,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6480,7 +6494,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6494,7 +6508,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6508,7 +6522,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6522,7 +6536,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6536,7 +6550,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6550,7 +6564,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6564,7 +6578,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6578,7 +6592,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6592,7 +6606,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6606,7 +6620,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6620,7 +6634,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6631,7 +6645,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6642,7 +6656,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6656,7 +6670,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6670,7 +6684,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6684,7 +6698,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6698,7 +6712,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6712,7 +6726,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6726,7 +6740,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6740,7 +6754,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6754,7 +6768,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6765,7 +6779,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6776,7 +6790,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6787,7 +6801,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6801,7 +6815,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6815,7 +6829,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -6829,7 +6843,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -6843,7 +6857,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -6857,60 +6871,74 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
       <c r="B194" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="C194">
+        <v>2.74</v>
       </c>
       <c r="D194">
-        <v>2.74</v>
-      </c>
-      <c r="E194">
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
       <c r="B195" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="C195">
+        <v>2.73</v>
       </c>
       <c r="D195">
-        <v>2.73</v>
-      </c>
-      <c r="E195">
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
       <c r="B196" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="C196">
+        <v>2.8</v>
       </c>
       <c r="D196">
-        <v>2.8</v>
-      </c>
-      <c r="E196">
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
       <c r="B197" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="C197">
+        <v>2.82</v>
       </c>
       <c r="D197">
-        <v>2.8</v>
-      </c>
-      <c r="E197">
-        <v>2.6</v>
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A198" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B198" t="s">
+        <v>61</v>
+      </c>
+      <c r="C198">
+        <v>2.85</v>
+      </c>
+      <c r="D198">
+        <v>2.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-08-07
NORMAL/SLOWING · GDPNow 5.83 · NY 2.24
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0174EF66-3B42-4D05-85A8-2C037002A395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12857E8-540E-4314-9E1B-BB2DFFFD7D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1604,15 +1604,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="5"/>
+    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1624,7 +1624,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1634,67 +1634,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
+    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +1703,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1712,14 +1712,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1737,55 +1737,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1794,7 +1794,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1803,13 +1803,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1841,14 +1841,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P198"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P199"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.1796875" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1857,7 +1857,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1869,16 +1869,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1976,7 +1976,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2169,7 +2169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2529,7 +2529,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2550,7 +2550,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2569,7 +2569,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2588,7 +2588,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2607,7 +2607,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2626,7 +2626,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2647,7 +2647,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2668,7 +2668,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2689,7 +2689,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2710,7 +2710,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2731,7 +2731,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2752,7 +2752,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2773,7 +2773,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2794,7 +2794,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2815,7 +2815,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2834,7 +2834,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2853,7 +2853,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2872,7 +2872,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2891,7 +2891,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2912,7 +2912,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2933,7 +2933,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2954,7 +2954,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2975,7 +2975,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2996,7 +2996,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3017,7 +3017,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3038,7 +3038,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3059,7 +3059,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3080,7 +3080,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3099,7 +3099,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3115,7 +3115,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3399,7 +3399,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3506,7 +3506,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3588,7 +3588,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3610,7 +3610,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3621,7 +3621,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3700,7 +3700,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3711,7 +3711,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3722,7 +3722,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3901,7 +3901,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3945,7 +3945,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3961,7 +3961,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3972,7 +3972,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3994,7 +3994,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4005,7 +4005,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4038,7 +4038,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -4117,7 +4117,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -4181,6 +4181,14 @@
       </c>
       <c r="P198">
         <v>2.52</v>
+      </c>
+    </row>
+    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A199" s="2">
+        <v>46241</v>
+      </c>
+      <c r="P199">
+        <v>2.2400000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -4204,18 +4212,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I198"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I199"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4224,7 +4232,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4236,16 +4244,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4262,7 +4270,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4273,7 +4281,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4284,7 +4292,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4295,7 +4303,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4306,7 +4314,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4317,7 +4325,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4328,7 +4336,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4339,7 +4347,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4350,7 +4358,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4361,7 +4369,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4372,7 +4380,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4383,7 +4391,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4394,7 +4402,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4408,7 +4416,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4422,7 +4430,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4436,7 +4444,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4450,7 +4458,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4464,7 +4472,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4478,7 +4486,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4492,7 +4500,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4506,7 +4514,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4520,7 +4528,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4534,7 +4542,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4545,7 +4553,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4556,7 +4564,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4567,7 +4575,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4581,7 +4589,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4595,7 +4603,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4609,7 +4617,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4623,7 +4631,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4637,7 +4645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4651,7 +4659,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4665,7 +4673,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4679,7 +4687,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4693,7 +4701,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4707,7 +4715,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4718,7 +4726,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4729,7 +4737,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4740,7 +4748,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4751,7 +4759,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4765,7 +4773,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4779,7 +4787,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4793,7 +4801,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4807,7 +4815,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4821,7 +4829,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4835,7 +4843,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4849,7 +4857,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4863,7 +4871,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4877,7 +4885,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4888,7 +4896,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4899,7 +4907,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4910,7 +4918,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4921,7 +4929,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -4935,7 +4943,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -4949,7 +4957,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -4963,7 +4971,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -4977,7 +4985,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -4991,7 +4999,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -5008,7 +5016,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -5025,7 +5033,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -5042,7 +5050,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -5059,7 +5067,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -5074,7 +5082,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5089,7 +5097,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5104,7 +5112,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5119,7 +5127,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5136,7 +5144,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5153,7 +5161,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5167,7 +5175,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5181,7 +5189,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5198,7 +5206,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5215,7 +5223,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5232,7 +5240,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5249,7 +5257,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5266,7 +5274,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5281,7 +5289,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5296,7 +5304,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5311,7 +5319,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5326,7 +5334,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5343,7 +5351,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5360,7 +5368,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5377,7 +5385,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5394,7 +5402,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5411,7 +5419,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5428,7 +5436,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5445,7 +5453,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5462,7 +5470,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5479,7 +5487,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5494,7 +5502,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5509,7 +5517,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5524,7 +5532,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5539,7 +5547,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5556,7 +5564,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5573,7 +5581,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5590,7 +5598,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5604,7 +5612,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5618,7 +5626,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5632,7 +5640,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5646,7 +5654,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5661,7 +5669,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5676,7 +5684,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5691,7 +5699,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5704,7 +5712,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5717,7 +5725,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5730,7 +5738,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5743,7 +5751,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5758,7 +5766,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5773,7 +5781,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5788,7 +5796,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5803,7 +5811,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5817,7 +5825,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5831,7 +5839,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5845,7 +5853,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5859,7 +5867,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5873,7 +5881,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5884,7 +5892,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5895,7 +5903,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5906,7 +5914,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5920,7 +5928,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5934,7 +5942,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -5948,7 +5956,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -5962,7 +5970,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -5976,7 +5984,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -5990,7 +5998,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -6004,7 +6012,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -6018,7 +6026,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -6032,7 +6040,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -6046,7 +6054,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -6057,7 +6065,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -6068,7 +6076,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -6079,7 +6087,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6093,7 +6101,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6107,7 +6115,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6121,7 +6129,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6136,7 +6144,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6151,7 +6159,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6165,7 +6173,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6180,7 +6188,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6195,7 +6203,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6210,7 +6218,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6225,7 +6233,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6238,7 +6246,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6251,7 +6259,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6264,7 +6272,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6279,7 +6287,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6294,7 +6302,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6309,7 +6317,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6323,7 +6331,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6337,7 +6345,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6351,7 +6359,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6365,7 +6373,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6379,7 +6387,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6393,7 +6401,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6407,7 +6415,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6421,7 +6429,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6435,7 +6443,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6449,7 +6457,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6466,7 +6474,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6480,7 +6488,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6494,7 +6502,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6508,7 +6516,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6522,7 +6530,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6536,7 +6544,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6550,7 +6558,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6564,7 +6572,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6578,7 +6586,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6592,7 +6600,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6606,7 +6614,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6620,7 +6628,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6634,7 +6642,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6645,7 +6653,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6656,7 +6664,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6670,7 +6678,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6684,7 +6692,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6698,7 +6706,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6712,7 +6720,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6726,7 +6734,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6740,7 +6748,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6754,7 +6762,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6768,7 +6776,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6779,7 +6787,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6790,7 +6798,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6801,7 +6809,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6815,7 +6823,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6829,7 +6837,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -6843,7 +6851,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -6857,7 +6865,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -6871,7 +6879,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -6885,7 +6893,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -6899,7 +6907,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -6913,7 +6921,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -6927,7 +6935,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -6939,6 +6947,17 @@
       </c>
       <c r="D198">
         <v>2.52</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" s="2">
+        <v>46241</v>
+      </c>
+      <c r="B199" t="s">
+        <v>61</v>
+      </c>
+      <c r="D199">
+        <v>2.2400000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-08-14
NORMAL/SLOWING · GDPNow 4.31 · NY 2.14
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12857E8-540E-4314-9E1B-BB2DFFFD7D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BA00C4-E3F7-45E4-A960-F1B2CFAE5413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P199"/>
+  <dimension ref="A1:P200"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -4189,6 +4189,14 @@
       </c>
       <c r="P199">
         <v>2.2400000000000002</v>
+      </c>
+    </row>
+    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A200" s="2">
+        <v>46248</v>
+      </c>
+      <c r="P200">
+        <v>2.14</v>
       </c>
     </row>
   </sheetData>
@@ -4212,7 +4220,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -6958,6 +6966,17 @@
       </c>
       <c r="D199">
         <v>2.2400000000000002</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" s="2">
+        <v>46248</v>
+      </c>
+      <c r="B200" t="s">
+        <v>61</v>
+      </c>
+      <c r="D200">
+        <v>2.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-08-21
NORMAL/SLOWING · GDPNow 4.03 · NY 2.27
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BA00C4-E3F7-45E4-A960-F1B2CFAE5413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A3814D-313C-4A0A-9A8D-BED95AF3AEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1006,6 +1006,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1017,9 +1020,6 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1613,26 +1613,26 @@
   <sheetData>
     <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
     </row>
     <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P200"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -1849,31 +1849,31 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
+      <c r="D4" s="33"/>
     </row>
     <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -4197,6 +4197,14 @@
       </c>
       <c r="P200">
         <v>2.14</v>
+      </c>
+    </row>
+    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A201" s="2">
+        <v>46255</v>
+      </c>
+      <c r="P201">
+        <v>2.27</v>
       </c>
     </row>
   </sheetData>
@@ -4220,7 +4228,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -4232,31 +4240,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
+      <c r="D4" s="33"/>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -6977,6 +6985,17 @@
       </c>
       <c r="D200">
         <v>2.14</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" s="2">
+        <v>46255</v>
+      </c>
+      <c r="B201" t="s">
+        <v>61</v>
+      </c>
+      <c r="D201">
+        <v>2.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-08-29
NORMAL/SLOWING · GDPNow 4.61 · NY 2.22
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A3814D-313C-4A0A-9A8D-BED95AF3AEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B6ECC8-E4C5-4B74-90D3-37CD0E99D39E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1006,9 +1006,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1020,6 +1017,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1613,26 +1613,26 @@
   <sheetData>
     <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
     </row>
     <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
     </row>
     <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P201"/>
+  <dimension ref="A1:P202"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -1849,31 +1849,31 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
+      <c r="D4" s="32"/>
     </row>
     <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -4205,6 +4205,14 @@
       </c>
       <c r="P201">
         <v>2.27</v>
+      </c>
+    </row>
+    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A202" s="2">
+        <v>46262</v>
+      </c>
+      <c r="P202">
+        <v>2.2200000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -4228,7 +4236,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:I202"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -4240,31 +4248,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="33"/>
+      <c r="D4" s="32"/>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
@@ -6996,6 +7004,17 @@
       </c>
       <c r="D201">
         <v>2.27</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" s="2">
+        <v>46262</v>
+      </c>
+      <c r="B202" t="s">
+        <v>61</v>
+      </c>
+      <c r="D202">
+        <v>2.2200000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-09-05
NORMAL/SLOWING · GDPNow 4.75 · NY 2.26
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B6ECC8-E4C5-4B74-90D3-37CD0E99D39E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C142E9D-8DAB-4E9A-A6FB-776E4380DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:P202"/>
+  <dimension ref="A1:Q203"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -4117,7 +4117,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -4183,7 +4183,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -4191,7 +4191,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -4207,12 +4207,23 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
       <c r="P202">
         <v>2.2200000000000002</v>
+      </c>
+    </row>
+    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A203" s="2">
+        <v>46269</v>
+      </c>
+      <c r="P203">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="Q203">
+        <v>2.5099999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -4236,7 +4247,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I202"/>
+  <dimension ref="A1:I203"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -7015,6 +7026,20 @@
       </c>
       <c r="D202">
         <v>2.2200000000000002</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B203" t="s">
+        <v>61</v>
+      </c>
+      <c r="D203">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="E203">
+        <v>2.5099999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>